<commit_message>
Bishop: Auto stock sync 1C: retry after transient GitHub commit_refs failure
</commit_message>
<xml_diff>
--- a/tma_static/data/Roastberry_Прайс_2026.xlsx
+++ b/tma_static/data/Roastberry_Прайс_2026.xlsx
@@ -10,8 +10,8 @@
     <sheet name="Прайс кофе" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Прайс кофе'!$A$5:$I$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Прайс кофе'!$A$1:$I$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Прайс кофе'!$A$5:$I$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Прайс кофе'!$A$1:$I$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Прайс кофе'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,12 +19,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="54">
   <si>
     <t>ПРАЙС КОФЕ ROASTBERRY</t>
   </si>
   <si>
-    <t>Обновлено 07.10.2026</t>
+    <t>Обновлено 24.08.2026</t>
   </si>
   <si>
     <t>Цены за упаковку · ₽ с НДС</t>
@@ -51,13 +51,13 @@
     <t>базовая 200 г</t>
   </si>
   <si>
-    <t>смеси</t>
+    <t>СМЕСИ</t>
   </si>
   <si>
     <t>CLASSICA #1</t>
   </si>
   <si>
-    <t>эспрессо</t>
+    <t>Эспрессо</t>
   </si>
   <si>
     <t>БИТТЕР</t>
@@ -72,10 +72,10 @@
     <t>ЛУНГО</t>
   </si>
   <si>
-    <t>фильтр</t>
-  </si>
-  <si>
-    <t>моносорта</t>
+    <t>Фильтр</t>
+  </si>
+  <si>
+    <t>МОНОСОРТА</t>
   </si>
   <si>
     <t>Бразилия Сан Рафаель</t>
@@ -90,7 +90,7 @@
     <t>Вьетнам Блю Шонла</t>
   </si>
   <si>
-    <t>фильтр, эспрессо</t>
+    <t>Фильтр, Эспрессо</t>
   </si>
   <si>
     <t>Гватемала Уэуэтенанго</t>
@@ -105,7 +105,7 @@
     <t>Кения АБ Центральная провинция</t>
   </si>
   <si>
-    <t>эспрессо, фильтр</t>
+    <t>Эспрессо, Фильтр</t>
   </si>
   <si>
     <t>Китай Симао Гр.1</t>
@@ -114,13 +114,13 @@
     <t>Колумбия Андино</t>
   </si>
   <si>
-    <t>Колумбия Рисаральда Декаф</t>
+    <t>Колумбия Риссальда Декаф</t>
   </si>
   <si>
     <t>Коста-Рика Тарразу</t>
   </si>
   <si>
-    <t>Никарагуа Марагаджип мытый</t>
+    <t>Никарагуа Марагаджип</t>
   </si>
   <si>
     <t>Перу гр.1</t>
@@ -144,10 +144,7 @@
     <t>Эфиопия Сидамо гр.2</t>
   </si>
   <si>
-    <t>Эфиопия Иргачиф гр.2</t>
-  </si>
-  <si>
-    <t>блэк</t>
+    <t>BLACK</t>
   </si>
   <si>
     <t>Кения Маакиоу Пиберри</t>
@@ -159,19 +156,16 @@
     <t>Эфиопия Банко Готити гр.1</t>
   </si>
   <si>
+    <t>—</t>
+  </si>
+  <si>
     <t>Эфиопия Конга гр.1</t>
   </si>
   <si>
-    <t>Индонезия Суматра Гайо Гр.1</t>
-  </si>
-  <si>
-    <t>Кения Оранж Кисии</t>
-  </si>
-  <si>
-    <t>борщ</t>
-  </si>
-  <si>
-    <t>Кения КиаваМуруру NH-7</t>
+    <t>BORЩ</t>
+  </si>
+  <si>
+    <t>Кения КиаваМуруру</t>
   </si>
   <si>
     <t>Колумбия Катимор</t>
@@ -186,10 +180,7 @@
     <t>Эфиопия Гедеб гр.1 Ананасовый настой</t>
   </si>
   <si>
-    <t>Эфиопия ВОРКА Челчеле гр.1 анаэроб.</t>
-  </si>
-  <si>
-    <t>Колумбия Арбуз Декаф</t>
+    <t>Эфиопия Челчеле гр.1</t>
   </si>
 </sst>
 </file>
@@ -423,13 +414,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1312259</xdr:colOff>
+      <xdr:colOff>1299313</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>229743</xdr:rowOff>
+      <xdr:rowOff>111081</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -446,8 +437,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="38100" y="9525"/>
-          <a:ext cx="2188559" cy="534543"/>
+          <a:off x="38100" y="47625"/>
+          <a:ext cx="2175613" cy="377781"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -747,7 +738,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -1320,22 +1311,22 @@
         <v>12</v>
       </c>
       <c r="D23" s="14">
-        <v>2860</v>
+        <v>2545</v>
       </c>
       <c r="E23" s="14">
-        <v>2575</v>
+        <v>2295</v>
       </c>
       <c r="F23" s="14">
-        <v>2290</v>
+        <v>2040</v>
       </c>
       <c r="G23" s="14">
-        <v>600</v>
+        <v>540</v>
       </c>
       <c r="H23" s="14">
-        <v>540</v>
+        <v>486</v>
       </c>
       <c r="I23" s="14">
-        <v>480</v>
+        <v>432</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="24" customHeight="1">
@@ -1433,7 +1424,7 @@
         <v>37</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="D27" s="14">
         <v>2070</v>
@@ -1523,432 +1514,316 @@
         <v>28</v>
       </c>
       <c r="D30" s="14">
-        <v>2230</v>
+        <v>2385</v>
       </c>
       <c r="E30" s="14">
-        <v>2010</v>
+        <v>2150</v>
       </c>
       <c r="F30" s="14">
-        <v>1785</v>
+        <v>1910</v>
       </c>
       <c r="G30" s="14">
-        <v>475</v>
+        <v>505</v>
       </c>
       <c r="H30" s="15">
-        <v>427.5</v>
+        <v>454.5</v>
       </c>
       <c r="I30" s="14">
-        <v>380</v>
+        <v>404</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="24" customHeight="1">
-      <c r="A31" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B31" s="12" t="s">
+      <c r="A31" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C31" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="D31" s="14">
-        <v>2335</v>
-      </c>
-      <c r="E31" s="14">
-        <v>2105</v>
-      </c>
-      <c r="F31" s="14">
-        <v>1870</v>
-      </c>
-      <c r="G31" s="14">
-        <v>495</v>
-      </c>
-      <c r="H31" s="15">
-        <v>445.5</v>
-      </c>
-      <c r="I31" s="14">
-        <v>396</v>
+      <c r="B31" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="9">
+        <v>2960</v>
+      </c>
+      <c r="E31" s="9">
+        <v>2665</v>
+      </c>
+      <c r="F31" s="9">
+        <v>2370</v>
+      </c>
+      <c r="G31" s="9">
+        <v>670</v>
+      </c>
+      <c r="H31" s="9">
+        <v>603</v>
+      </c>
+      <c r="I31" s="9">
+        <v>540</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="24" customHeight="1">
-      <c r="A32" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="B32" s="7" t="s">
+      <c r="A32" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D32" s="9">
-        <v>2960</v>
-      </c>
-      <c r="E32" s="9">
-        <v>2665</v>
-      </c>
-      <c r="F32" s="9">
-        <v>2370</v>
-      </c>
-      <c r="G32" s="9">
-        <v>670</v>
-      </c>
-      <c r="H32" s="9">
-        <v>603</v>
-      </c>
-      <c r="I32" s="9">
-        <v>540</v>
+      <c r="D32" s="15">
+        <v>2847.5</v>
+      </c>
+      <c r="E32" s="14">
+        <v>2565</v>
+      </c>
+      <c r="F32" s="14">
+        <v>2280</v>
+      </c>
+      <c r="G32" s="14">
+        <v>650</v>
+      </c>
+      <c r="H32" s="14">
+        <v>585</v>
+      </c>
+      <c r="I32" s="14">
+        <v>520</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="24" customHeight="1">
       <c r="A33" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B33" s="12" t="s">
         <v>44</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D33" s="15">
-        <v>2847.5</v>
+        <v>45</v>
+      </c>
+      <c r="D33" s="14">
+        <v>3020</v>
       </c>
       <c r="E33" s="14">
-        <v>2565</v>
+        <v>2720</v>
       </c>
       <c r="F33" s="14">
-        <v>2280</v>
+        <v>2420</v>
       </c>
       <c r="G33" s="14">
-        <v>650</v>
-      </c>
-      <c r="H33" s="14">
-        <v>585</v>
+        <v>685</v>
+      </c>
+      <c r="H33" s="15">
+        <v>616.5</v>
       </c>
       <c r="I33" s="14">
-        <v>520</v>
+        <v>550</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="24" customHeight="1">
       <c r="A34" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>17</v>
       </c>
       <c r="D34" s="14">
-        <v>3020</v>
+        <v>2945</v>
       </c>
       <c r="E34" s="14">
-        <v>2720</v>
+        <v>2655</v>
       </c>
       <c r="F34" s="14">
-        <v>2420</v>
+        <v>2360</v>
       </c>
       <c r="G34" s="14">
-        <v>685</v>
-      </c>
-      <c r="H34" s="15">
-        <v>616.5</v>
+        <v>670</v>
+      </c>
+      <c r="H34" s="14">
+        <v>603</v>
       </c>
       <c r="I34" s="14">
-        <v>550</v>
+        <v>540</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="24" customHeight="1">
-      <c r="A35" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C35" s="13" t="s">
+      <c r="A35" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D35" s="14">
-        <v>2945</v>
-      </c>
-      <c r="E35" s="14">
-        <v>2655</v>
-      </c>
-      <c r="F35" s="14">
-        <v>2360</v>
-      </c>
-      <c r="G35" s="14">
-        <v>670</v>
-      </c>
-      <c r="H35" s="14">
-        <v>603</v>
-      </c>
-      <c r="I35" s="14">
-        <v>540</v>
+      <c r="D35" s="10">
+        <v>3972.5</v>
+      </c>
+      <c r="E35" s="9">
+        <v>3580</v>
+      </c>
+      <c r="F35" s="9">
+        <v>3180</v>
+      </c>
+      <c r="G35" s="9">
+        <v>875</v>
+      </c>
+      <c r="H35" s="10">
+        <v>787.5</v>
+      </c>
+      <c r="I35" s="9">
+        <v>700</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="24" customHeight="1">
-      <c r="A36" s="19" t="s">
-        <v>42</v>
+      <c r="A36" s="21" t="s">
+        <v>47</v>
       </c>
       <c r="B36" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="15">
+        <v>4602.5</v>
+      </c>
+      <c r="E36" s="14">
+        <v>4145</v>
+      </c>
+      <c r="F36" s="14">
+        <v>3685</v>
+      </c>
+      <c r="G36" s="14">
+        <v>1000</v>
+      </c>
+      <c r="H36" s="14">
+        <v>900</v>
+      </c>
+      <c r="I36" s="14">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="24" customHeight="1">
+      <c r="A37" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C36" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D36" s="14">
-        <v>2465</v>
-      </c>
-      <c r="E36" s="14">
-        <v>2220</v>
-      </c>
-      <c r="F36" s="14">
-        <v>1975</v>
-      </c>
-      <c r="G36" s="14">
-        <v>575</v>
-      </c>
-      <c r="H36" s="15">
-        <v>517.5</v>
-      </c>
-      <c r="I36" s="14">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="24" customHeight="1">
-      <c r="A37" s="19" t="s">
-        <v>42</v>
-      </c>
       <c r="B37" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="D37" s="15">
-        <v>2067.5</v>
+        <v>4602.5</v>
       </c>
       <c r="E37" s="14">
-        <v>1865</v>
+        <v>4145</v>
       </c>
       <c r="F37" s="14">
-        <v>1655</v>
+        <v>3685</v>
       </c>
       <c r="G37" s="14">
-        <v>495</v>
-      </c>
-      <c r="H37" s="15">
-        <v>445.5</v>
+        <v>1000</v>
+      </c>
+      <c r="H37" s="14">
+        <v>900</v>
       </c>
       <c r="I37" s="14">
-        <v>400</v>
+        <v>800</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="24" customHeight="1">
-      <c r="A38" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="B38" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C38" s="8" t="s">
+      <c r="A38" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C38" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D38" s="10">
-        <v>3972.5</v>
-      </c>
-      <c r="E38" s="9">
-        <v>3580</v>
-      </c>
-      <c r="F38" s="9">
-        <v>3180</v>
-      </c>
-      <c r="G38" s="9">
-        <v>875</v>
-      </c>
-      <c r="H38" s="10">
-        <v>787.5</v>
-      </c>
-      <c r="I38" s="9">
-        <v>700</v>
+      <c r="D38" s="15">
+        <v>5922.5</v>
+      </c>
+      <c r="E38" s="14">
+        <v>5335</v>
+      </c>
+      <c r="F38" s="14">
+        <v>4740</v>
+      </c>
+      <c r="G38" s="14">
+        <v>1265</v>
+      </c>
+      <c r="H38" s="15">
+        <v>1138.5</v>
+      </c>
+      <c r="I38" s="14">
+        <v>1015</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="24" customHeight="1">
       <c r="A39" s="21" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C39" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D39" s="15">
-        <v>4602.5</v>
+      <c r="D39" s="14">
+        <v>3020</v>
       </c>
       <c r="E39" s="14">
-        <v>4145</v>
+        <v>2720</v>
       </c>
       <c r="F39" s="14">
-        <v>3685</v>
+        <v>2420</v>
       </c>
       <c r="G39" s="14">
-        <v>1000</v>
-      </c>
-      <c r="H39" s="14">
-        <v>900</v>
+        <v>685</v>
+      </c>
+      <c r="H39" s="15">
+        <v>616.5</v>
       </c>
       <c r="I39" s="14">
-        <v>800</v>
+        <v>550</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="24" customHeight="1">
       <c r="A40" s="21" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D40" s="15">
-        <v>4602.5</v>
+        <v>23</v>
+      </c>
+      <c r="D40" s="14">
+        <v>3020</v>
       </c>
       <c r="E40" s="14">
-        <v>4145</v>
+        <v>2720</v>
       </c>
       <c r="F40" s="14">
-        <v>3685</v>
+        <v>2420</v>
       </c>
       <c r="G40" s="14">
-        <v>1000</v>
-      </c>
-      <c r="H40" s="14">
-        <v>900</v>
+        <v>685</v>
+      </c>
+      <c r="H40" s="15">
+        <v>616.5</v>
       </c>
       <c r="I40" s="14">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="24" customHeight="1">
-      <c r="A41" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B41" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="C41" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D41" s="15">
-        <v>5922.5</v>
-      </c>
-      <c r="E41" s="14">
-        <v>5335</v>
-      </c>
-      <c r="F41" s="14">
-        <v>4740</v>
-      </c>
-      <c r="G41" s="14">
-        <v>1265</v>
-      </c>
-      <c r="H41" s="15">
-        <v>1138.5</v>
-      </c>
-      <c r="I41" s="14">
-        <v>1015</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="24" customHeight="1">
-      <c r="A42" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D42" s="14">
-        <v>3020</v>
-      </c>
-      <c r="E42" s="14">
-        <v>2720</v>
-      </c>
-      <c r="F42" s="14">
-        <v>2420</v>
-      </c>
-      <c r="G42" s="14">
-        <v>685</v>
-      </c>
-      <c r="H42" s="15">
-        <v>616.5</v>
-      </c>
-      <c r="I42" s="14">
         <v>550</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="24" customHeight="1">
-      <c r="A43" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D43" s="14">
-        <v>3020</v>
-      </c>
-      <c r="E43" s="14">
-        <v>2720</v>
-      </c>
-      <c r="F43" s="14">
-        <v>2420</v>
-      </c>
-      <c r="G43" s="14">
-        <v>685</v>
-      </c>
-      <c r="H43" s="15">
-        <v>616.5</v>
-      </c>
-      <c r="I43" s="14">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="24" customHeight="1">
-      <c r="A44" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="C44" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D44" s="14">
-        <v>4130</v>
-      </c>
-      <c r="E44" s="14">
-        <v>3720</v>
-      </c>
-      <c r="F44" s="14">
-        <v>3305</v>
-      </c>
-      <c r="G44" s="14">
-        <v>905</v>
-      </c>
-      <c r="H44" s="15">
-        <v>814.5</v>
-      </c>
-      <c r="I44" s="14">
-        <v>725</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:I44"/>
+  <autoFilter ref="A5:I40"/>
   <mergeCells count="3">
     <mergeCell ref="D1:I1"/>
     <mergeCell ref="D2:I2"/>

</xml_diff>

<commit_message>
Bishop: Auto stock sync from 1C: stock updates 246
</commit_message>
<xml_diff>
--- a/tma_static/data/Roastberry_Прайс_2026.xlsx
+++ b/tma_static/data/Roastberry_Прайс_2026.xlsx
@@ -10,8 +10,8 @@
     <sheet name="прайс" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">прайс!$A$5:$I$48</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">прайс!$A$1:$H$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">прайс!$A$5:$I$50</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">прайс!$A$1:$H$52</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">прайс!$4:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,12 +19,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="67">
   <si>
     <t>roastberry · прайс-лист</t>
   </si>
   <si>
-    <t>Действует с 01.07.2026 · обновлено 07.10.2026</t>
+    <t>Действует с 01.07.2026 · обновлено 16.10.2026</t>
   </si>
   <si>
     <t>цены за упаковку, ₽ с НДС · скидки 10% от 10 кг, 20% от 25 кг</t>
@@ -84,7 +84,7 @@
     <t>BF</t>
   </si>
   <si>
-    <t>моносорта · 21 позиция</t>
+    <t>моносорта · 23 позиции</t>
   </si>
   <si>
     <t>моносорта</t>
@@ -162,9 +162,15 @@
     <t>Эфиопия Сидамо гр.2</t>
   </si>
   <si>
+    <t>Эфиопия Milk · новинка</t>
+  </si>
+  <si>
     <t>Эфиопия Иргачиф гр.2</t>
   </si>
   <si>
+    <t>Эфиопия Сидамо Гр.4 · новинка</t>
+  </si>
+  <si>
     <t>BLACK Edition · 85+ SCA · 6 позиций</t>
   </si>
   <si>
@@ -183,7 +189,7 @@
     <t>Эфиопия Конга гр.1</t>
   </si>
   <si>
-    <t>Индонезия Суматра Гайо Гр.1 · новинка</t>
+    <t>Индонезия Суматра Гайо Гр.1</t>
   </si>
   <si>
     <t>Кения Оранж Кисии · новинка</t>
@@ -737,7 +743,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
@@ -1574,101 +1580,101 @@
         <v>46</v>
       </c>
       <c r="B33" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C33" s="13">
+        <v>2015</v>
+      </c>
+      <c r="D33" s="14">
+        <v>1815</v>
+      </c>
+      <c r="E33" s="14">
+        <v>1615</v>
+      </c>
+      <c r="F33" s="15">
+        <v>435</v>
+      </c>
+      <c r="G33" s="16">
+        <v>391.5</v>
+      </c>
+      <c r="H33" s="14">
+        <v>348</v>
+      </c>
+      <c r="I33" s="17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="18" customHeight="1">
+      <c r="A34" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="C33" s="13">
+      <c r="C34" s="13">
         <v>2335</v>
       </c>
-      <c r="D33" s="14">
+      <c r="D34" s="14">
         <v>2105</v>
       </c>
-      <c r="E33" s="14">
+      <c r="E34" s="14">
         <v>1870</v>
       </c>
-      <c r="F33" s="15">
+      <c r="F34" s="15">
         <v>495</v>
       </c>
-      <c r="G33" s="16">
+      <c r="G34" s="16">
         <v>445.5</v>
       </c>
-      <c r="H33" s="14">
+      <c r="H34" s="14">
         <v>396</v>
       </c>
-      <c r="I33" s="17" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="22" customHeight="1">
-      <c r="A34" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="B34" s="19"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="19" t="s">
-        <v>48</v>
+      <c r="I34" s="17" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="18" customHeight="1">
       <c r="A35" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C35" s="13">
+        <v>2015</v>
+      </c>
+      <c r="D35" s="14">
+        <v>1815</v>
+      </c>
+      <c r="E35" s="14">
+        <v>1615</v>
+      </c>
+      <c r="F35" s="15">
+        <v>435</v>
+      </c>
+      <c r="G35" s="16">
+        <v>391.5</v>
+      </c>
+      <c r="H35" s="14">
+        <v>348</v>
+      </c>
+      <c r="I35" s="17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="22" customHeight="1">
+      <c r="A36" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B35" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C35" s="13">
-        <v>2960</v>
-      </c>
-      <c r="D35" s="14">
-        <v>2665</v>
-      </c>
-      <c r="E35" s="14">
-        <v>2370</v>
-      </c>
-      <c r="F35" s="15">
-        <v>670</v>
-      </c>
-      <c r="G35" s="16">
-        <v>603</v>
-      </c>
-      <c r="H35" s="14">
-        <v>540</v>
-      </c>
-      <c r="I35" s="17" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="18" customHeight="1">
-      <c r="A36" s="11" t="s">
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="19"/>
+      <c r="G36" s="19"/>
+      <c r="H36" s="19"/>
+      <c r="I36" s="19" t="s">
         <v>50</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C36" s="13">
-        <v>2847.5</v>
-      </c>
-      <c r="D36" s="14">
-        <v>2565</v>
-      </c>
-      <c r="E36" s="14">
-        <v>2280</v>
-      </c>
-      <c r="F36" s="15">
-        <v>650</v>
-      </c>
-      <c r="G36" s="16">
-        <v>585</v>
-      </c>
-      <c r="H36" s="14">
-        <v>520</v>
-      </c>
-      <c r="I36" s="17" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="18" customHeight="1">
@@ -1679,25 +1685,25 @@
         <v>25</v>
       </c>
       <c r="C37" s="13">
-        <v>3020</v>
+        <v>2960</v>
       </c>
       <c r="D37" s="14">
-        <v>2720</v>
+        <v>2665</v>
       </c>
       <c r="E37" s="14">
-        <v>2420</v>
+        <v>2370</v>
       </c>
       <c r="F37" s="15">
-        <v>685</v>
+        <v>670</v>
       </c>
       <c r="G37" s="16">
-        <v>616.5</v>
+        <v>603</v>
       </c>
       <c r="H37" s="14">
-        <v>550</v>
+        <v>540</v>
       </c>
       <c r="I37" s="17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="18" customHeight="1">
@@ -1708,25 +1714,25 @@
         <v>25</v>
       </c>
       <c r="C38" s="13">
-        <v>2945</v>
+        <v>2847.5</v>
       </c>
       <c r="D38" s="14">
-        <v>2655</v>
+        <v>2565</v>
       </c>
       <c r="E38" s="14">
-        <v>2360</v>
+        <v>2280</v>
       </c>
       <c r="F38" s="15">
-        <v>670</v>
+        <v>650</v>
       </c>
       <c r="G38" s="16">
-        <v>603</v>
+        <v>585</v>
       </c>
       <c r="H38" s="14">
-        <v>540</v>
+        <v>520</v>
       </c>
       <c r="I38" s="17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="18" customHeight="1">
@@ -1734,28 +1740,28 @@
         <v>53</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C39" s="13">
-        <v>2465</v>
+        <v>3020</v>
       </c>
       <c r="D39" s="14">
-        <v>2220</v>
+        <v>2720</v>
       </c>
       <c r="E39" s="14">
-        <v>1975</v>
+        <v>2420</v>
       </c>
       <c r="F39" s="15">
-        <v>575</v>
+        <v>685</v>
       </c>
       <c r="G39" s="16">
-        <v>517.5</v>
+        <v>616.5</v>
       </c>
       <c r="H39" s="14">
-        <v>460</v>
+        <v>550</v>
       </c>
       <c r="I39" s="17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="18" customHeight="1">
@@ -1763,101 +1769,101 @@
         <v>54</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C40" s="13">
-        <v>2067.5</v>
+        <v>2945</v>
       </c>
       <c r="D40" s="14">
-        <v>1865</v>
+        <v>2655</v>
       </c>
       <c r="E40" s="14">
-        <v>1655</v>
+        <v>2360</v>
       </c>
       <c r="F40" s="15">
-        <v>495</v>
+        <v>670</v>
       </c>
       <c r="G40" s="16">
-        <v>445.5</v>
+        <v>603</v>
       </c>
       <c r="H40" s="14">
-        <v>400</v>
+        <v>540</v>
       </c>
       <c r="I40" s="17" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="22" customHeight="1">
-      <c r="A41" s="20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="18" customHeight="1">
+      <c r="A41" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B41" s="21"/>
-      <c r="C41" s="21"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="21"/>
-      <c r="F41" s="21"/>
-      <c r="G41" s="21"/>
-      <c r="H41" s="21"/>
-      <c r="I41" s="21" t="s">
-        <v>56</v>
+      <c r="B41" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C41" s="13">
+        <v>2465</v>
+      </c>
+      <c r="D41" s="14">
+        <v>2220</v>
+      </c>
+      <c r="E41" s="14">
+        <v>1975</v>
+      </c>
+      <c r="F41" s="15">
+        <v>575</v>
+      </c>
+      <c r="G41" s="16">
+        <v>517.5</v>
+      </c>
+      <c r="H41" s="14">
+        <v>460</v>
+      </c>
+      <c r="I41" s="17" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="18" customHeight="1">
       <c r="A42" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C42" s="13">
+        <v>2067.5</v>
+      </c>
+      <c r="D42" s="14">
+        <v>1865</v>
+      </c>
+      <c r="E42" s="14">
+        <v>1655</v>
+      </c>
+      <c r="F42" s="15">
+        <v>495</v>
+      </c>
+      <c r="G42" s="16">
+        <v>445.5</v>
+      </c>
+      <c r="H42" s="14">
+        <v>400</v>
+      </c>
+      <c r="I42" s="17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="22" customHeight="1">
+      <c r="A43" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="B42" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C42" s="13">
-        <v>3972.5</v>
-      </c>
-      <c r="D42" s="14">
-        <v>3580</v>
-      </c>
-      <c r="E42" s="14">
-        <v>3180</v>
-      </c>
-      <c r="F42" s="15">
-        <v>875</v>
-      </c>
-      <c r="G42" s="16">
-        <v>787.5</v>
-      </c>
-      <c r="H42" s="14">
-        <v>700</v>
-      </c>
-      <c r="I42" s="17" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="18" customHeight="1">
-      <c r="A43" s="11" t="s">
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="21"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="21"/>
+      <c r="G43" s="21"/>
+      <c r="H43" s="21"/>
+      <c r="I43" s="21" t="s">
         <v>58</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C43" s="13">
-        <v>4602.5</v>
-      </c>
-      <c r="D43" s="14">
-        <v>4145</v>
-      </c>
-      <c r="E43" s="14">
-        <v>3685</v>
-      </c>
-      <c r="F43" s="15">
-        <v>1000</v>
-      </c>
-      <c r="G43" s="16">
-        <v>900</v>
-      </c>
-      <c r="H43" s="14">
-        <v>800</v>
-      </c>
-      <c r="I43" s="17" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="18" customHeight="1">
@@ -1868,25 +1874,25 @@
         <v>25</v>
       </c>
       <c r="C44" s="13">
-        <v>4602.5</v>
+        <v>3972.5</v>
       </c>
       <c r="D44" s="14">
-        <v>4145</v>
+        <v>3580</v>
       </c>
       <c r="E44" s="14">
-        <v>3685</v>
+        <v>3180</v>
       </c>
       <c r="F44" s="15">
-        <v>1000</v>
+        <v>875</v>
       </c>
       <c r="G44" s="16">
-        <v>900</v>
+        <v>787.5</v>
       </c>
       <c r="H44" s="14">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="I44" s="17" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="18" customHeight="1">
@@ -1897,25 +1903,25 @@
         <v>25</v>
       </c>
       <c r="C45" s="13">
-        <v>5922.5</v>
+        <v>4602.5</v>
       </c>
       <c r="D45" s="14">
-        <v>5335</v>
+        <v>4145</v>
       </c>
       <c r="E45" s="14">
-        <v>4740</v>
+        <v>3685</v>
       </c>
       <c r="F45" s="15">
-        <v>1265</v>
+        <v>1000</v>
       </c>
       <c r="G45" s="16">
-        <v>1138.5</v>
+        <v>900</v>
       </c>
       <c r="H45" s="14">
-        <v>1015</v>
+        <v>800</v>
       </c>
       <c r="I45" s="17" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="18" customHeight="1">
@@ -1926,25 +1932,25 @@
         <v>25</v>
       </c>
       <c r="C46" s="13">
-        <v>3020</v>
+        <v>4602.5</v>
       </c>
       <c r="D46" s="14">
-        <v>2720</v>
+        <v>4145</v>
       </c>
       <c r="E46" s="14">
-        <v>2420</v>
+        <v>3685</v>
       </c>
       <c r="F46" s="15">
-        <v>685</v>
+        <v>1000</v>
       </c>
       <c r="G46" s="16">
-        <v>616.5</v>
+        <v>900</v>
       </c>
       <c r="H46" s="14">
-        <v>550</v>
+        <v>800</v>
       </c>
       <c r="I46" s="17" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="18" customHeight="1">
@@ -1952,28 +1958,28 @@
         <v>62</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C47" s="13">
-        <v>3020</v>
+        <v>5922.5</v>
       </c>
       <c r="D47" s="14">
-        <v>2720</v>
+        <v>5335</v>
       </c>
       <c r="E47" s="14">
-        <v>2420</v>
+        <v>4740</v>
       </c>
       <c r="F47" s="15">
-        <v>685</v>
+        <v>1265</v>
       </c>
       <c r="G47" s="16">
-        <v>616.5</v>
+        <v>1138.5</v>
       </c>
       <c r="H47" s="14">
-        <v>550</v>
+        <v>1015</v>
       </c>
       <c r="I47" s="17" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="18" customHeight="1">
@@ -1984,34 +1990,92 @@
         <v>25</v>
       </c>
       <c r="C48" s="13">
+        <v>3020</v>
+      </c>
+      <c r="D48" s="14">
+        <v>2720</v>
+      </c>
+      <c r="E48" s="14">
+        <v>2420</v>
+      </c>
+      <c r="F48" s="15">
+        <v>685</v>
+      </c>
+      <c r="G48" s="16">
+        <v>616.5</v>
+      </c>
+      <c r="H48" s="14">
+        <v>550</v>
+      </c>
+      <c r="I48" s="17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="18" customHeight="1">
+      <c r="A49" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B49" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C49" s="13">
+        <v>3020</v>
+      </c>
+      <c r="D49" s="14">
+        <v>2720</v>
+      </c>
+      <c r="E49" s="14">
+        <v>2420</v>
+      </c>
+      <c r="F49" s="15">
+        <v>685</v>
+      </c>
+      <c r="G49" s="16">
+        <v>616.5</v>
+      </c>
+      <c r="H49" s="14">
+        <v>550</v>
+      </c>
+      <c r="I49" s="17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="18" customHeight="1">
+      <c r="A50" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B50" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C50" s="13">
         <v>4130</v>
       </c>
-      <c r="D48" s="14">
+      <c r="D50" s="14">
         <v>3720</v>
       </c>
-      <c r="E48" s="14">
+      <c r="E50" s="14">
         <v>3305</v>
       </c>
-      <c r="F48" s="15">
+      <c r="F50" s="15">
         <v>905</v>
       </c>
-      <c r="G48" s="16">
+      <c r="G50" s="16">
         <v>814.5</v>
       </c>
-      <c r="H48" s="14">
+      <c r="H50" s="14">
         <v>725</v>
       </c>
-      <c r="I48" s="17" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1">
-      <c r="A50" s="22" t="s">
-        <v>64</v>
+      <c r="I50" s="17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="22" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I48"/>
+  <autoFilter ref="A5:I50"/>
   <mergeCells count="3">
     <mergeCell ref="C1:H1"/>
     <mergeCell ref="C4:E4"/>

</xml_diff>

<commit_message>
Bishop: RBO hourly refresh: Main warehouse, Base price
</commit_message>
<xml_diff>
--- a/tma_static/data/Roastberry_Прайс_2026.xlsx
+++ b/tma_static/data/Roastberry_Прайс_2026.xlsx
@@ -10,8 +10,8 @@
     <sheet name="прайс" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">прайс!$A$5:$I$50</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">прайс!$A$1:$H$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">прайс!$A$5:$I$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">прайс!$A$1:$H$53</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">прайс!$4:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,12 +19,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="68">
   <si>
     <t>roastberry · прайс-лист</t>
   </si>
   <si>
-    <t>Действует с 01.07.2026 · обновлено 16.10.2026</t>
+    <t>Действует с 01.07.2026 · обновлено 25.10.2026</t>
   </si>
   <si>
     <t>цены за упаковку, ₽ с НДС · скидки 10% от 10 кг, 20% от 25 кг</t>
@@ -198,7 +198,7 @@
 новинка</t>
   </si>
   <si>
-    <t>BORЩ Edition · эксперимент · 7 позиций</t>
+    <t>BORЩ Edition · эксперимент · 8 позиций</t>
   </si>
   <si>
     <t>BORЩ Edition</t>
@@ -223,6 +223,10 @@
   </si>
   <si>
     <t>Колумбия Арбуз Декаф</t>
+  </si>
+  <si>
+    <t>Уганда Момо Бит бочка
+новинка</t>
   </si>
   <si>
     <t>+7 (995) 690-00-77 · Telegram @rbr_zakaz · roastberry.coffee · Пермь, ул. Деревообделочная, 8к6</t>
@@ -749,7 +753,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
@@ -2075,13 +2079,42 @@
         <v>58</v>
       </c>
     </row>
-    <row r="52" spans="1:9">
-      <c r="A52" s="23" t="s">
+    <row r="51" spans="1:9" ht="33" customHeight="1">
+      <c r="A51" s="18" t="s">
         <v>66</v>
       </c>
+      <c r="B51" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C51" s="13">
+        <v>3657.5</v>
+      </c>
+      <c r="D51" s="14">
+        <v>3295</v>
+      </c>
+      <c r="E51" s="14">
+        <v>2930</v>
+      </c>
+      <c r="F51" s="15">
+        <v>810</v>
+      </c>
+      <c r="G51" s="16">
+        <v>729</v>
+      </c>
+      <c r="H51" s="14">
+        <v>650</v>
+      </c>
+      <c r="I51" s="17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="23" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I50"/>
+  <autoFilter ref="A5:I51"/>
   <mergeCells count="3">
     <mergeCell ref="C1:H1"/>
     <mergeCell ref="C4:E4"/>

</xml_diff>